<commit_message>
Add three federal cases missing from the September 21 dataset.
Podrybau, Doverspike, and Whitney showed up in a comparison with CaseLinker and were not in the workbook.
</commit_message>
<xml_diff>
--- a/Pfefferkorn & Demeocq - AI-CSAM Prosecutions Dataset (2026-09-21).xlsx
+++ b/Pfefferkorn & Demeocq - AI-CSAM Prosecutions Dataset (2026-09-21).xlsx
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1362" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1375" uniqueCount="484">
   <si>
     <t>Title</t>
   </si>
@@ -1572,6 +1572,42 @@
   <si>
     <t>Outcome 
 (as of 9/21/2026)</t>
+  </si>
+  <si>
+    <t>U.S. v. Podrybau</t>
+  </si>
+  <si>
+    <t>5:25-cr-40027</t>
+  </si>
+  <si>
+    <t>https://www.courtlistener.com/docket/70264285/united-states-v-podrybau/</t>
+  </si>
+  <si>
+    <t>Plea (sentencing 11/17/2026)</t>
+  </si>
+  <si>
+    <t>U.S. v. Doverspike</t>
+  </si>
+  <si>
+    <t>6:23-cr-03083</t>
+  </si>
+  <si>
+    <t>U.S. v. Whitney</t>
+  </si>
+  <si>
+    <t>1:23-cr-00124</t>
+  </si>
+  <si>
+    <t>E.D. Va.</t>
+  </si>
+  <si>
+    <t>18 U.S.C. §§ 2252(a)(2), 1466A(a)(1), 2252(a)(4)(B)</t>
+  </si>
+  <si>
+    <t>https://www.courtlistener.com/docket/67740132/united-states-v-doverspike/</t>
+  </si>
+  <si>
+    <t>https://www.courtlistener.com/docket/67648912/united-states-v-whitney/</t>
   </si>
 </sst>
 </file>
@@ -6944,6 +6980,171 @@
       <c r="V72" s="3"/>
       <c r="W72" s="3"/>
     </row>
+    <row r="73" spans="1:23" ht="13" x14ac:dyDescent="0.15">
+      <c r="A73" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E73" s="5">
+        <v>45777</v>
+      </c>
+      <c r="F73" s="3">
+        <v>2025</v>
+      </c>
+      <c r="G73" s="3"/>
+      <c r="H73" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="I73" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J73" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K73" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L73" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="M73" s="3"/>
+      <c r="N73" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O73" s="3"/>
+      <c r="P73" s="3"/>
+      <c r="Q73" s="3"/>
+      <c r="R73" s="3"/>
+      <c r="S73" s="3"/>
+      <c r="T73" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="U73" s="3"/>
+      <c r="V73" s="3"/>
+      <c r="W73" s="3"/>
+    </row>
+    <row r="74" spans="1:23" ht="13" x14ac:dyDescent="0.15">
+      <c r="A74" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="E74" s="5">
+        <v>45167</v>
+      </c>
+      <c r="F74" s="3">
+        <v>2023</v>
+      </c>
+      <c r="G74" s="3"/>
+      <c r="H74" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="I74" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J74" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K74" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L74" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="M74" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="N74" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O74" s="3"/>
+      <c r="P74" s="3"/>
+      <c r="Q74" s="3"/>
+      <c r="R74" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="S74" s="3"/>
+      <c r="T74" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="U74" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="V74" s="3"/>
+      <c r="W74" s="3"/>
+    </row>
+    <row r="75" spans="1:23" ht="13" x14ac:dyDescent="0.15">
+      <c r="A75" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="E75" s="5">
+        <v>45134</v>
+      </c>
+      <c r="F75" s="3">
+        <v>2023</v>
+      </c>
+      <c r="G75" s="3"/>
+      <c r="H75" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="I75" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="J75" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K75" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L75" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="M75" s="3"/>
+      <c r="N75" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O75" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="P75" s="3"/>
+      <c r="Q75" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R75" s="3"/>
+      <c r="S75" s="3"/>
+      <c r="T75" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="U75" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="V75" s="3"/>
+      <c r="W75" s="3"/>
+    </row>
     <row r="85" spans="1:12" ht="13" x14ac:dyDescent="0.15">
       <c r="E85" s="5"/>
       <c r="I85" s="7"/>
@@ -10128,6 +10329,9 @@
     <hyperlink ref="L71" r:id="rId86" xr:uid="{46030B60-B2D7-7F42-BDE1-3775DC6E74A6}"/>
     <hyperlink ref="L72" r:id="rId87" xr:uid="{44756F98-98DA-3A4D-8D59-8B0C0AB72BF6}"/>
     <hyperlink ref="R60" r:id="rId88" location="docket" xr:uid="{074A3C58-17B2-A349-8396-2028F34BBAB5}"/>
+    <hyperlink ref="L73" r:id="rId93" xr:uid="{8CC32C7F-C87B-412D-B873-94C38A47DF23}"/>
+    <hyperlink ref="L74" r:id="rId94" xr:uid="{FA1D26A8-0040-4948-B358-0807E5FA5661}"/>
+    <hyperlink ref="L75" r:id="rId95" xr:uid="{E9011639-C5C5-414D-8285-7216909BCC07}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId89"/>

</xml_diff>

<commit_message>
Add Erselius and Sanders, flagged from press releases that say the material was AI-generated.
</commit_message>
<xml_diff>
--- a/Pfefferkorn & Demeocq - AI-CSAM Prosecutions Dataset (2026-09-21).xlsx
+++ b/Pfefferkorn & Demeocq - AI-CSAM Prosecutions Dataset (2026-09-21).xlsx
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1375" uniqueCount="484">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="492">
   <si>
     <t>Title</t>
   </si>
@@ -1608,6 +1608,30 @@
   </si>
   <si>
     <t>https://www.courtlistener.com/docket/67648912/united-states-v-whitney/</t>
+  </si>
+  <si>
+    <t>U.S. v. Erselius</t>
+  </si>
+  <si>
+    <t>3:25-cr-00070</t>
+  </si>
+  <si>
+    <t>18 U.S.C. §§ 2252A(a)(2), 2261A</t>
+  </si>
+  <si>
+    <t>https://www.courtlistener.com/docket/71599385/united-states-v-erselius/</t>
+  </si>
+  <si>
+    <t>U.S. v. Sanders</t>
+  </si>
+  <si>
+    <t>4:26-cr-00117</t>
+  </si>
+  <si>
+    <t>https://www.courtlistener.com/docket/73152226/united-states-v-sanders/</t>
+  </si>
+  <si>
+    <t>Convicted</t>
   </si>
 </sst>
 </file>
@@ -7145,6 +7169,63 @@
       <c r="V75" s="3"/>
       <c r="W75" s="3"/>
     </row>
+    <row r="76" spans="1:23" ht="13" x14ac:dyDescent="0.15">
+      <c r="A76" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E76" s="5">
+        <v>45918</v>
+      </c>
+      <c r="F76" s="3">
+        <v>2025</v>
+      </c>
+      <c r="G76" s="3"/>
+      <c r="H76" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="I76" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J76" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="K76" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L76" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="M76" s="3"/>
+      <c r="N76" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O76" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="P76" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q76" s="3"/>
+      <c r="R76" s="3"/>
+      <c r="S76" s="3"/>
+      <c r="T76" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="U76" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="V76" s="3"/>
+      <c r="W76" s="3"/>
+    </row>
     <row r="85" spans="1:12" ht="13" x14ac:dyDescent="0.15">
       <c r="E85" s="5"/>
       <c r="I85" s="7"/>
@@ -10332,6 +10413,7 @@
     <hyperlink ref="L73" r:id="rId93" xr:uid="{8CC32C7F-C87B-412D-B873-94C38A47DF23}"/>
     <hyperlink ref="L74" r:id="rId94" xr:uid="{FA1D26A8-0040-4948-B358-0807E5FA5661}"/>
     <hyperlink ref="L75" r:id="rId95" xr:uid="{E9011639-C5C5-414D-8285-7216909BCC07}"/>
+    <hyperlink ref="L76" r:id="rId96" xr:uid="{7C2A1E40-6B14-4F2A-9C31-0A5D8E2F14B6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId89"/>
@@ -10341,7 +10423,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF7F658B-AEA7-7B48-8CE1-7C74ED7CFEE1}">
-  <dimension ref="A1:AK14"/>
+  <dimension ref="A1:AK15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="17.1640625" bestFit="1" customWidth="1"/>
@@ -11440,6 +11522,67 @@
       <c r="AJ14" s="10"/>
       <c r="AK14" s="10"/>
     </row>
+    <row r="15" spans="1:37" s="13" customFormat="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="10" t="s">
+        <v>488</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>489</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="E15" s="11">
+        <v>46118</v>
+      </c>
+      <c r="F15" s="10">
+        <v>2026</v>
+      </c>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="12" t="s">
+        <v>490</v>
+      </c>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="O15" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="P15" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10" t="s">
+        <v>491</v>
+      </c>
+      <c r="U15" s="10"/>
+      <c r="V15" s="10"/>
+      <c r="W15" s="10"/>
+      <c r="X15" s="10"/>
+      <c r="Y15" s="10"/>
+      <c r="Z15" s="10"/>
+      <c r="AA15" s="10"/>
+      <c r="AB15" s="10"/>
+      <c r="AC15" s="10"/>
+      <c r="AD15" s="10"/>
+      <c r="AE15" s="10"/>
+      <c r="AF15" s="10"/>
+      <c r="AG15" s="10"/>
+      <c r="AH15" s="10"/>
+      <c r="AI15" s="10"/>
+      <c r="AJ15" s="10"/>
+      <c r="AK15" s="10"/>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="L2" r:id="rId1" xr:uid="{1B427427-0FEE-6040-A702-04F33540370A}"/>
@@ -11456,6 +11599,7 @@
     <hyperlink ref="L11" r:id="rId12" xr:uid="{2DA09326-B584-0148-B0BA-9CC5ED135A0A}"/>
     <hyperlink ref="L13" r:id="rId13" xr:uid="{4976269A-3A1C-0B49-B2E3-730BA089B655}"/>
     <hyperlink ref="L14" r:id="rId14" xr:uid="{10938D43-FA0D-D44A-840E-981AF7F65B64}"/>
+    <hyperlink ref="L15" r:id="rId15" xr:uid="{3E8B0C71-2D44-4A19-B6F0-91C4A7D25E18}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>